<commit_message>
Final Required Function Version
</commit_message>
<xml_diff>
--- a/hardware/amr_pin_mapping_template.xlsx
+++ b/hardware/amr_pin_mapping_template.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="331">
   <si>
     <t>Module Type</t>
   </si>
@@ -208,6 +208,44 @@
   </si>
   <si>
     <t>PG0</t>
+  </si>
+  <si>
+    <r>
+      <t>Ultrasonic 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>右边</t>
+    </r>
+  </si>
+  <si>
+    <t>PC7</t>
+  </si>
+  <si>
+    <t>PC5</t>
+  </si>
+  <si>
+    <r>
+      <t>Ultrasonic 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>左边</t>
+    </r>
+  </si>
+  <si>
+    <t>PA6</t>
+  </si>
+  <si>
+    <t>PA3</t>
   </si>
   <si>
     <t>Board Pin Number</t>
@@ -1015,7 +1053,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1178,6 +1216,11 @@
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="34">
@@ -1649,10 +1692,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2186,7 +2230,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="3" width="16" customWidth="1"/>
@@ -2957,6 +3001,146 @@
       </c>
       <c r="H24">
         <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="2">
+        <v>30</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="2">
+        <v>32</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="2">
+        <v>28</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="2">
+        <v>25</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -2978,54 +3162,54 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>14</v>
@@ -3033,43 +3217,43 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>14</v>
@@ -3077,10 +3261,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>14</v>
@@ -3088,7 +3272,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>46</v>
@@ -3099,7 +3283,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>47</v>
@@ -3110,32 +3294,32 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="2" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>14</v>
@@ -3143,142 +3327,142 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="2" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>14</v>
@@ -3286,10 +3470,10 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>14</v>
@@ -3297,10 +3481,10 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>14</v>
@@ -3308,18 +3492,18 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="2" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>46</v>
@@ -3330,7 +3514,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="2" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>47</v>
@@ -3341,164 +3525,164 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="2" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="2" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="2" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="2" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="2" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="2" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="2" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="2" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="2" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="2" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="2" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="2" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="2" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>14</v>
@@ -3506,10 +3690,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="2" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>14</v>
@@ -3517,10 +3701,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="2" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>14</v>
@@ -3528,128 +3712,128 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="2" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="2" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="2" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="2" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="2" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="2" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="2" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="2" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="2" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="2" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="2" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>46</v>
@@ -3660,7 +3844,7 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="2" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>47</v>
@@ -3671,32 +3855,32 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="2" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="2" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="2" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>14</v>
@@ -3704,10 +3888,10 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="2" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>14</v>
@@ -3715,10 +3899,10 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" s="2" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>14</v>
@@ -3726,10 +3910,10 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="2" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>14</v>
@@ -3737,10 +3921,10 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="2" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>14</v>
@@ -3748,109 +3932,109 @@
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="2" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" s="2" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" s="2" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" s="2" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" s="2" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" s="2" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" s="2" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="2" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" s="2" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" s="2" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>14</v>
@@ -3858,7 +4042,7 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" s="2" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>46</v>
@@ -3869,7 +4053,7 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" s="2" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>47</v>
@@ -3880,194 +4064,194 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" s="2" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" s="2" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="2" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" s="2" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" s="2" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" s="2" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" s="2" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" s="2" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" s="2" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" s="2" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" s="2" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" s="2" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" s="2" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" s="2" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" s="2" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" s="2" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" s="2" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>47</v>
@@ -4078,10 +4262,10 @@
     </row>
     <row r="101" spans="1:3">
       <c r="A101" s="2" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>46</v>

</xml_diff>